<commit_message>
Started refactor according to Clean Architecture requirements: -created folders domain, application, infrastructure, presentation -transfered buiseness logic to domain -created use_cases based on specific brands implementations -created file_io for file managing and scrapers for selenium based web scrapers implementation -modified function driven aproach to class implementation
</commit_message>
<xml_diff>
--- a/for_client/Claas_AS_20.01.26.xlsx_quotation.xlsx
+++ b/for_client/Claas_AS_20.01.26.xlsx_quotation.xlsx
@@ -413,259 +413,226 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>codes</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>qty</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Qty</t>
+          <t>monthly_prices</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Weekly</t>
+          <t>weekly_prices</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1234002</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1234002</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
           <t>1</t>
         </is>
       </c>
+      <c r="C2" t="n">
+        <v>131.51733408</v>
+      </c>
       <c r="D2" t="n">
-        <v>131.51733408</v>
-      </c>
-      <c r="E2" t="n">
         <v>165.71787408</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1365171</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1365171</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
           <t>1</t>
         </is>
       </c>
+      <c r="C3" t="n">
+        <v>41.00458032</v>
+      </c>
       <c r="D3" t="n">
-        <v>41.00458032</v>
-      </c>
-      <c r="E3" t="n">
         <v>48.32134032</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>22833652</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>22833652</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
           <t>1</t>
         </is>
       </c>
+      <c r="C4" t="n">
+        <v>1597.08971268</v>
+      </c>
       <c r="D4" t="n">
-        <v>1597.08971268</v>
-      </c>
-      <c r="E4" t="n">
         <v>2013.52265268</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2355210</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2355210</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
           <t>4</t>
         </is>
       </c>
+      <c r="C5" t="n">
+        <v>0.45743412</v>
+      </c>
       <c r="D5" t="n">
-        <v>0.45743412</v>
-      </c>
-      <c r="E5" t="n">
         <v>0.5333341200000001</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2368280</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2368280</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
           <t>8</t>
         </is>
       </c>
+      <c r="C6" t="n">
+        <v>0.3403356</v>
+      </c>
       <c r="D6" t="n">
-        <v>0.3403356</v>
-      </c>
-      <c r="E6" t="n">
         <v>0.4314156</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1253750</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1253750</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
           <t>2</t>
         </is>
       </c>
+      <c r="C7" t="n">
+        <v>10.53956508</v>
+      </c>
       <c r="D7" t="n">
-        <v>10.53956508</v>
-      </c>
-      <c r="E7" t="n">
         <v>13.36304508</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1238521</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1238521</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
           <t>4</t>
         </is>
       </c>
+      <c r="C8" t="n">
+        <v>3.934655999999999</v>
+      </c>
       <c r="D8" t="n">
-        <v>3.934655999999999</v>
-      </c>
-      <c r="E8" t="n">
         <v>4.648116</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1253041</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1253041</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
           <t>1</t>
         </is>
       </c>
+      <c r="C9" t="n">
+        <v>63.21841548</v>
+      </c>
       <c r="D9" t="n">
-        <v>63.21841548</v>
-      </c>
-      <c r="E9" t="n">
         <v>80.18965548</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1430830</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1430830</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
           <t>4</t>
         </is>
       </c>
+      <c r="C10" t="n">
+        <v>2.49972096</v>
+      </c>
       <c r="D10" t="n">
-        <v>2.49972096</v>
-      </c>
-      <c r="E10" t="n">
         <v>3.16764096</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8475600</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>8475600</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
           <t>12</t>
         </is>
       </c>
+      <c r="C11" t="n">
+        <v>6.71171556</v>
+      </c>
       <c r="D11" t="n">
-        <v>6.71171556</v>
-      </c>
-      <c r="E11" t="n">
         <v>8.533315559999998</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>10</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2381320</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2381320</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
           <t>4</t>
         </is>
       </c>
+      <c r="C12" t="n">
+        <v>0.21634536</v>
+      </c>
       <c r="D12" t="n">
-        <v>0.21634536</v>
-      </c>
-      <c r="E12" t="n">
         <v>0.26188536</v>
       </c>
     </row>

</xml_diff>